<commit_message>
Add search_menu tool: find drinks by ingredient
</commit_message>
<xml_diff>
--- a/data/menu.xlsx
+++ b/data/menu.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
   <si>
     <t>напиток</t>
   </si>
@@ -22,28 +22,151 @@
     <t>время_приготовления_мин</t>
   </si>
   <si>
+    <t>состав</t>
+  </si>
+  <si>
     <t>эспрессо</t>
   </si>
   <si>
+    <t>кофе</t>
+  </si>
+  <si>
     <t>американо</t>
   </si>
   <si>
+    <t>кофе, вода</t>
+  </si>
+  <si>
     <t>капучино</t>
   </si>
   <si>
+    <t>кофе, молоко, молочная пена</t>
+  </si>
+  <si>
     <t>латте</t>
   </si>
   <si>
-    <t>раф</t>
+    <t>кофе, молоко</t>
   </si>
   <si>
     <t>флэт уайт</t>
   </si>
   <si>
-    <t>чай</t>
-  </si>
-  <si>
-    <t>какао</t>
+    <t>раф классический</t>
+  </si>
+  <si>
+    <t>кофе, сливки, ванильный сироп</t>
+  </si>
+  <si>
+    <t>Баунти</t>
+  </si>
+  <si>
+    <t>кофе, кокосовое молоко, кокосовый сироп</t>
+  </si>
+  <si>
+    <t>Кокосовый бриз</t>
+  </si>
+  <si>
+    <t>кокосовый сироп, газированная вода, лёд</t>
+  </si>
+  <si>
+    <t>Кокосовый риф</t>
+  </si>
+  <si>
+    <t>кофе, сливки, кокосовый сироп</t>
+  </si>
+  <si>
+    <t>Белый пляж</t>
+  </si>
+  <si>
+    <t>кокосовое молоко, ванильное мороженое, кокосовый сироп</t>
+  </si>
+  <si>
+    <t>Розовый закат</t>
+  </si>
+  <si>
+    <t>кофе, молоко, арбузный сироп</t>
+  </si>
+  <si>
+    <t>Розовая волна</t>
+  </si>
+  <si>
+    <t>арбузный сироп, газированная вода, лёд</t>
+  </si>
+  <si>
+    <t>Арбузный смузи</t>
+  </si>
+  <si>
+    <t>арбузный сироп, лёд, мята</t>
+  </si>
+  <si>
+    <t>Марципан</t>
+  </si>
+  <si>
+    <t>кофе, миндальное молоко</t>
+  </si>
+  <si>
+    <t>Амаретто латте</t>
+  </si>
+  <si>
+    <t>кофе, молоко, миндальный сироп</t>
+  </si>
+  <si>
+    <t>Миндальное облако</t>
+  </si>
+  <si>
+    <t>кофе, сливки, миндальный сироп</t>
+  </si>
+  <si>
+    <t>Облако</t>
+  </si>
+  <si>
+    <t>Карамельный латте</t>
+  </si>
+  <si>
+    <t>кофе, молоко, карамельный сироп</t>
+  </si>
+  <si>
+    <t>Изумруд</t>
+  </si>
+  <si>
+    <t>матча, молоко</t>
+  </si>
+  <si>
+    <t>Сладкоежка</t>
+  </si>
+  <si>
+    <t>какао, молоко</t>
+  </si>
+  <si>
+    <t>Трюфель</t>
+  </si>
+  <si>
+    <t>шоколад, молоко, сливки</t>
+  </si>
+  <si>
+    <t>Зелёный дракон</t>
+  </si>
+  <si>
+    <t>зелёный чай</t>
+  </si>
+  <si>
+    <t>Тропик</t>
+  </si>
+  <si>
+    <t>маракуйя, ананасовый сироп, газированная вода</t>
+  </si>
+  <si>
+    <t>Лесная ягода</t>
+  </si>
+  <si>
+    <t>малиновый сироп, газированная вода, лёд</t>
+  </si>
+  <si>
+    <t>Цитрус</t>
+  </si>
+  <si>
+    <t>апельсиновый сироп, лимон, газированная вода</t>
   </si>
 </sst>
 </file>
@@ -420,10 +543,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -433,10 +556,13 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>120</v>
@@ -444,10 +570,13 @@
       <c r="C2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B3">
         <v>140</v>
@@ -455,10 +584,13 @@
       <c r="C3">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>180</v>
@@ -466,10 +598,13 @@
       <c r="C4">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>200</v>
@@ -477,49 +612,302 @@
       <c r="C5">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B6">
+        <v>210</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
         <v>220</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
-        <v>210</v>
-      </c>
-      <c r="C7">
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>240</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>260</v>
+      </c>
+      <c r="C9">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10">
+        <v>250</v>
+      </c>
+      <c r="C10">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11">
+        <v>280</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12">
+        <v>230</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13">
+        <v>260</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14">
+        <v>270</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15">
+        <v>240</v>
+      </c>
+      <c r="C15">
+        <v>5</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16">
+        <v>250</v>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17">
+        <v>250</v>
+      </c>
+      <c r="C17">
+        <v>6</v>
+      </c>
+      <c r="D17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18">
+        <v>220</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19">
+        <v>230</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>250</v>
+      </c>
+      <c r="C20">
+        <v>5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21">
+        <v>170</v>
+      </c>
+      <c r="C21">
+        <v>5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22">
+        <v>230</v>
+      </c>
+      <c r="C22">
+        <v>6</v>
+      </c>
+      <c r="D22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23">
         <v>100</v>
       </c>
-      <c r="C8">
+      <c r="C23">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>170</v>
-      </c>
-      <c r="C9">
-        <v>5</v>
+      <c r="D23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24">
+        <v>260</v>
+      </c>
+      <c r="C24">
+        <v>4</v>
+      </c>
+      <c r="D24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25">
+        <v>250</v>
+      </c>
+      <c r="C25">
+        <v>4</v>
+      </c>
+      <c r="D25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26">
+        <v>240</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+      <c r="D26" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>